<commit_message>
add base boosting stuff to the repo
</commit_message>
<xml_diff>
--- a/results/benchmark_results.xlsx
+++ b/results/benchmark_results.xlsx
@@ -4082,18 +4082,14 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>mae</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>0.435</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>0.011</v>
       </c>
     </row>
     <row r="3">
@@ -4119,18 +4115,14 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>0.945</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>0.007</v>
       </c>
     </row>
     <row r="4">
@@ -4156,18 +4148,14 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>0.931</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>0.005</v>
       </c>
     </row>
     <row r="5">
@@ -4193,18 +4181,14 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>0.718</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>0.025</v>
       </c>
     </row>
     <row r="6">
@@ -4230,18 +4214,14 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>mae</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>0.627</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>0.002</v>
       </c>
     </row>
     <row r="7">
@@ -4267,18 +4247,14 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>mae</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>0.004</v>
       </c>
     </row>
     <row r="8">
@@ -4304,18 +4280,14 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>0.008999999999999999</v>
       </c>
     </row>
     <row r="9">
@@ -4341,18 +4313,14 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>mae</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>8.797000000000001</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>0.06900000000000001</v>
       </c>
     </row>
     <row r="10">
@@ -4378,18 +4346,14 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>spearman</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>0.454</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>0.031</v>
       </c>
     </row>
     <row r="11">
@@ -4415,18 +4379,14 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>pr-auc</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>0.663</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>0.004</v>
       </c>
     </row>
     <row r="12">
@@ -4452,18 +4412,14 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>pr-auc</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>0.858</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>0.001</v>
       </c>
     </row>
     <row r="13">
@@ -4489,18 +4445,14 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>pr-auc</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>0.779</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>0.002</v>
       </c>
     </row>
     <row r="14">
@@ -4526,18 +4478,14 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>pr-auc</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>0.424</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>0.023</v>
       </c>
     </row>
     <row r="15">
@@ -4563,18 +4511,14 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>pr-auc</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>0.713</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>0.006</v>
       </c>
     </row>
     <row r="16">
@@ -4600,18 +4544,14 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G16" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>0.649</v>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>0.01</v>
       </c>
     </row>
     <row r="17">
@@ -4637,18 +4577,14 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>spearman</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>0.383</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>0.027</v>
       </c>
     </row>
     <row r="18">
@@ -4674,18 +4610,14 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>spearman</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>0.017</v>
       </c>
     </row>
     <row r="19">
@@ -4711,18 +4643,14 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>spearman</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="n">
+        <v>0.592</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>0.008999999999999999</v>
       </c>
     </row>
     <row r="20">
@@ -4748,18 +4676,14 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>mae</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>0.658</v>
+      </c>
+      <c r="G20" s="3" t="n">
+        <v>0.001</v>
       </c>
     </row>
     <row r="21">
@@ -4785,18 +4709,14 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>0.828</v>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>0.01</v>
       </c>
     </row>
     <row r="22">
@@ -4822,18 +4742,14 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G22" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="n">
+        <v>0.824</v>
+      </c>
+      <c r="G22" s="3" t="n">
+        <v>0.005</v>
       </c>
     </row>
     <row r="23">
@@ -4859,18 +4775,14 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G23" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="n">
+        <v>0.901</v>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>0.008</v>
       </c>
     </row>
   </sheetData>
@@ -4956,18 +4868,14 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>mae</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>0.421</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>0.026</v>
       </c>
     </row>
     <row r="3">
@@ -4993,18 +4901,14 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>0.9419999999999999</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>0.013</v>
       </c>
     </row>
     <row r="4">
@@ -5030,18 +4934,14 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>0.915</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>0.008999999999999999</v>
       </c>
     </row>
     <row r="5">
@@ -5067,18 +4967,14 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>0.031</v>
       </c>
     </row>
     <row r="6">
@@ -5104,18 +5000,14 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>mae</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>0.704</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>0.012</v>
       </c>
     </row>
     <row r="7">
@@ -5141,18 +5033,14 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>mae</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>1.275</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>0.011</v>
       </c>
     </row>
     <row r="8">
@@ -5178,18 +5066,14 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>0.867</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>0.006</v>
       </c>
     </row>
     <row r="9">
@@ -5215,18 +5099,14 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>mae</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>9.943</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>0.063</v>
       </c>
     </row>
     <row r="10">
@@ -5252,18 +5132,14 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>spearman</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>0.475</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>0.03</v>
       </c>
     </row>
     <row r="11">
@@ -5289,18 +5165,14 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>pr-auc</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>0.026</v>
       </c>
     </row>
     <row r="12">
@@ -5326,18 +5198,14 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>pr-auc</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>0.835</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>0.007</v>
       </c>
     </row>
     <row r="13">
@@ -5363,18 +5231,14 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>pr-auc</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>0.733</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>0.003</v>
       </c>
     </row>
     <row r="14">
@@ -5400,18 +5264,14 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>pr-auc</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>0.377</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>0.016</v>
       </c>
     </row>
     <row r="15">
@@ -5437,18 +5297,14 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>pr-auc</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>0.649</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>0.023</v>
       </c>
     </row>
     <row r="16">
@@ -5474,18 +5330,14 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G16" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>0.634</v>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>0.01</v>
       </c>
     </row>
     <row r="17">
@@ -5511,18 +5363,14 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>spearman</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>0.399</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>0.051</v>
       </c>
     </row>
     <row r="18">
@@ -5548,18 +5396,14 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>spearman</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>0.273</v>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>0.008999999999999999</v>
       </c>
     </row>
     <row r="19">
@@ -5585,18 +5429,14 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>spearman</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>0.008</v>
       </c>
     </row>
     <row r="20">
@@ -5622,18 +5462,14 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>mae</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>0.633</v>
+      </c>
+      <c r="G20" s="3" t="n">
+        <v>0.012</v>
       </c>
     </row>
     <row r="21">
@@ -5659,18 +5495,14 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>0.762</v>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>0.023</v>
       </c>
     </row>
     <row r="22">
@@ -5696,18 +5528,14 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G22" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="n">
+        <v>0.835</v>
+      </c>
+      <c r="G22" s="3" t="n">
+        <v>0.007</v>
       </c>
     </row>
     <row r="23">
@@ -5733,18 +5561,14 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G23" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="n">
+        <v>0.844</v>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>0.03</v>
       </c>
     </row>
   </sheetData>
@@ -5830,18 +5654,14 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>mae</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>0.295</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>0.004</v>
       </c>
     </row>
     <row r="3">
@@ -5867,18 +5687,14 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>0.988</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>0.002</v>
       </c>
     </row>
     <row r="4">
@@ -5904,18 +5720,14 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>0.9340000000000001</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>0.001</v>
       </c>
     </row>
     <row r="5">
@@ -5941,18 +5753,14 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>0.726</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>0.005</v>
       </c>
     </row>
     <row r="6">
@@ -5978,18 +5786,14 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>mae</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>0.471</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>0.003</v>
       </c>
     </row>
     <row r="7">
@@ -6015,18 +5819,14 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>mae</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>0.861</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>0.01</v>
       </c>
     </row>
     <row r="8">
@@ -6052,18 +5852,14 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>0.894</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>0.002</v>
       </c>
     </row>
     <row r="9">
@@ -6089,18 +5885,14 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>mae</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>7.528</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>0.046</v>
       </c>
     </row>
     <row r="10">
@@ -6126,18 +5918,14 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>spearman</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>0.544</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>0.013</v>
       </c>
     </row>
     <row r="11">
@@ -6163,18 +5951,14 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>pr-auc</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>0.782</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>0.007</v>
       </c>
     </row>
     <row r="12">
@@ -6200,18 +5984,14 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>pr-auc</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>0.916</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>0.001</v>
       </c>
     </row>
     <row r="13">
@@ -6237,18 +6017,14 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>pr-auc</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>0.861</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>0.004</v>
       </c>
     </row>
     <row r="14">
@@ -6274,18 +6050,14 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>pr-auc</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>0.015</v>
       </c>
     </row>
     <row r="15">
@@ -6311,18 +6083,14 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>pr-auc</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>0.717</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>0.006</v>
       </c>
     </row>
     <row r="16">
@@ -6348,18 +6116,14 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G16" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>0.641</v>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>0.008999999999999999</v>
       </c>
     </row>
     <row r="17">
@@ -6385,18 +6149,14 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>spearman</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>0.027</v>
       </c>
     </row>
     <row r="18">
@@ -6422,18 +6182,14 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>spearman</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>0.513</v>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>0.019</v>
       </c>
     </row>
     <row r="19">
@@ -6459,18 +6215,14 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>spearman</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="n">
+        <v>0.583</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>0.021</v>
       </c>
     </row>
     <row r="20">
@@ -6496,18 +6248,14 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>mae</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>0.597</v>
+      </c>
+      <c r="G20" s="3" t="n">
+        <v>0.004</v>
       </c>
     </row>
     <row r="21">
@@ -6533,18 +6281,14 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>0.869</v>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>0.004</v>
       </c>
     </row>
     <row r="22">
@@ -6570,18 +6314,14 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G22" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="G22" s="3" t="n">
+        <v>0.003</v>
       </c>
     </row>
     <row r="23">
@@ -6607,18 +6347,14 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G23" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="n">
+        <v>0.9340000000000001</v>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>0.005</v>
       </c>
     </row>
   </sheetData>
@@ -6704,18 +6440,14 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>mae</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>0.422</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>0.032</v>
       </c>
     </row>
     <row r="3">
@@ -6741,18 +6473,14 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>0.987</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>0.002</v>
       </c>
     </row>
     <row r="4">
@@ -6778,18 +6506,14 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>0.9350000000000001</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>0.005</v>
       </c>
     </row>
     <row r="5">
@@ -6815,18 +6539,14 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>0.709</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>0.027</v>
       </c>
     </row>
     <row r="6">
@@ -6852,18 +6572,14 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>mae</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>0.538</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>0.008999999999999999</v>
       </c>
     </row>
     <row r="7">
@@ -6889,18 +6605,14 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>mae</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>1.002</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>0.024</v>
       </c>
     </row>
     <row r="8">
@@ -6926,18 +6638,14 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>0.911</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>0.006</v>
       </c>
     </row>
     <row r="9">
@@ -6963,18 +6671,14 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>mae</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>9.061999999999999</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>0.239</v>
       </c>
     </row>
     <row r="10">
@@ -7000,18 +6704,14 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>spearman</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>0.554</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>0.013</v>
       </c>
     </row>
     <row r="11">
@@ -7037,18 +6737,14 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>pr-auc</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>0.754</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>0.001</v>
       </c>
     </row>
     <row r="12">
@@ -7074,18 +6770,14 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>pr-auc</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>0.911</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>0.001</v>
       </c>
     </row>
     <row r="13">
@@ -7111,18 +6803,14 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>pr-auc</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>0.002</v>
       </c>
     </row>
     <row r="14">
@@ -7148,18 +6836,14 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>pr-auc</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>0.443</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>0.032</v>
       </c>
     </row>
     <row r="15">
@@ -7185,18 +6869,14 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>pr-auc</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>0.738</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>0.016</v>
       </c>
     </row>
     <row r="16">
@@ -7222,18 +6902,14 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G16" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>0.011</v>
       </c>
     </row>
     <row r="17">
@@ -7259,18 +6935,14 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>spearman</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>0.186</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>0.202</v>
       </c>
     </row>
     <row r="18">
@@ -7296,18 +6968,14 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>spearman</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>0.419</v>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>0.019</v>
       </c>
     </row>
     <row r="19">
@@ -7333,18 +7001,14 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>spearman</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="n">
+        <v>0.612</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>0.014</v>
       </c>
     </row>
     <row r="20">
@@ -7370,18 +7034,14 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>mae</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>0.661</v>
+      </c>
+      <c r="G20" s="3" t="n">
+        <v>0.026</v>
       </c>
     </row>
     <row r="21">
@@ -7407,18 +7067,14 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>0.829</v>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>0.011</v>
       </c>
     </row>
     <row r="22">
@@ -7444,18 +7100,14 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G22" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="n">
+        <v>0.851</v>
+      </c>
+      <c r="G22" s="3" t="n">
+        <v>0.005</v>
       </c>
     </row>
     <row r="23">
@@ -7481,18 +7133,14 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G23" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="n">
+        <v>0.9320000000000001</v>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>0.008</v>
       </c>
     </row>
   </sheetData>
@@ -7578,18 +7226,14 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>mae</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>0.346</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>0.006</v>
       </c>
     </row>
     <row r="3">
@@ -7615,18 +7259,14 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>0.985</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>0.002</v>
       </c>
     </row>
     <row r="4">
@@ -7652,18 +7292,14 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>0.906</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>0.003</v>
       </c>
     </row>
     <row r="5">
@@ -7689,18 +7325,14 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>0.681</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>0.025</v>
       </c>
     </row>
     <row r="6">
@@ -7726,18 +7358,14 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>mae</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>0.517</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>0.017</v>
       </c>
     </row>
     <row r="7">
@@ -7763,18 +7391,14 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>mae</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>0.766</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>0.021</v>
       </c>
     </row>
     <row r="8">
@@ -7800,18 +7424,14 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>0.902</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>0.004</v>
       </c>
     </row>
     <row r="9">
@@ -7837,18 +7457,14 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>mae</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>8.612</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>0.654</v>
       </c>
     </row>
     <row r="10">
@@ -7874,18 +7490,14 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>spearman</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>0.302</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>0.172</v>
       </c>
     </row>
     <row r="11">
@@ -8442,7 +8054,7 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Best of 10 sklearn/XGBoost models on 31 RDKit descriptors</t>
+          <t>ExtraTrees</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -8452,18 +8064,14 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>mae</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>0.353</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>0.083</v>
       </c>
     </row>
     <row r="3">
@@ -8479,7 +8087,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Best of 10 sklearn/XGBoost models on 31 RDKit descriptors</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -8489,18 +8097,14 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>0.922</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>0.006</v>
       </c>
     </row>
     <row r="4">
@@ -8516,7 +8120,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Best of 10 sklearn/XGBoost models on 31 RDKit descriptors</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -8526,18 +8130,14 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>0.884</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>0.008</v>
       </c>
     </row>
     <row r="5">
@@ -8553,7 +8153,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Best of 10 sklearn/XGBoost models on 31 RDKit descriptors</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -8563,18 +8163,14 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>0.676</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>0.012</v>
       </c>
     </row>
     <row r="6">
@@ -8590,7 +8186,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Best of 10 sklearn/XGBoost models on 31 RDKit descriptors</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -8600,18 +8196,14 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>mae</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>0.004</v>
       </c>
     </row>
     <row r="7">
@@ -8627,7 +8219,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Best of 10 sklearn/XGBoost models on 31 RDKit descriptors</t>
+          <t>ExtraTrees</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -8637,18 +8229,14 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>mae</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>0.834</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>0.011</v>
       </c>
     </row>
     <row r="8">
@@ -8664,7 +8252,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Best of 10 sklearn/XGBoost models on 31 RDKit descriptors</t>
+          <t>AdaBoost</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -8674,18 +8262,14 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>0.017</v>
       </c>
     </row>
     <row r="9">
@@ -8701,7 +8285,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Best of 10 sklearn/XGBoost models on 31 RDKit descriptors</t>
+          <t>AdaBoost</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -8711,18 +8295,14 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>mae</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>9.037000000000001</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>0.276</v>
       </c>
     </row>
     <row r="10">
@@ -8738,7 +8318,7 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Best of 10 sklearn/XGBoost models on 31 RDKit descriptors</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -8748,18 +8328,14 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>spearman</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>0.482</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>0.014</v>
       </c>
     </row>
     <row r="11">

</xml_diff>

<commit_message>
updated the runbencmark script for caliciboost; instead of the 2d and 3d padel descriptors, i decided to use only the 2d rdkit descriptors, which are more stable and less computationally expensive.; also updated the csv benchmark result files to include attentivefp and basicml results
</commit_message>
<xml_diff>
--- a/results/benchmark_results.xlsx
+++ b/results/benchmark_results.xlsx
@@ -7523,18 +7523,14 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>pr-auc</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>0.008</v>
       </c>
     </row>
     <row r="12">
@@ -7560,18 +7556,14 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>pr-auc</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>0.855</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>0.003</v>
       </c>
     </row>
     <row r="13">
@@ -7597,18 +7589,14 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>pr-auc</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>0.764</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>0.015</v>
       </c>
     </row>
     <row r="14">
@@ -7634,18 +7622,14 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>pr-auc</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>0.482</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>0.007</v>
       </c>
     </row>
     <row r="15">
@@ -7671,18 +7655,14 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>pr-auc</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>0.589</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>0.025</v>
       </c>
     </row>
     <row r="16">
@@ -7708,18 +7688,14 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G16" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>0.598</v>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>0.011</v>
       </c>
     </row>
     <row r="17">
@@ -7745,18 +7721,14 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>spearman</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>0.039</v>
       </c>
     </row>
     <row r="18">
@@ -7782,18 +7754,14 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>spearman</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>0.259</v>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>0.039</v>
       </c>
     </row>
     <row r="19">
@@ -7819,18 +7787,14 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>spearman</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="n">
+        <v>0.469</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>0.023</v>
       </c>
     </row>
     <row r="20">
@@ -7856,18 +7820,14 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>mae</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>0.631</v>
+      </c>
+      <c r="G20" s="3" t="n">
+        <v>0.024</v>
       </c>
     </row>
     <row r="21">
@@ -7893,18 +7853,14 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>0.839</v>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>0.007</v>
       </c>
     </row>
     <row r="22">
@@ -7930,18 +7886,14 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G22" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="n">
+        <v>0.831</v>
+      </c>
+      <c r="G22" s="3" t="n">
+        <v>0.004</v>
       </c>
     </row>
     <row r="23">
@@ -7967,18 +7919,14 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G23" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="n">
+        <v>0.914</v>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>0.007</v>
       </c>
     </row>
   </sheetData>
@@ -8351,7 +8299,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Best of 10 sklearn/XGBoost models on 31 RDKit descriptors</t>
+          <t>ExtraTrees</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -8361,18 +8309,14 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>pr-auc</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>0.603</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>0.021</v>
       </c>
     </row>
     <row r="12">
@@ -8388,7 +8332,7 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Best of 10 sklearn/XGBoost models on 31 RDKit descriptors</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -8398,18 +8342,14 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>pr-auc</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>0.801</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>0.003</v>
       </c>
     </row>
     <row r="13">
@@ -8425,7 +8365,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Best of 10 sklearn/XGBoost models on 31 RDKit descriptors</t>
+          <t>Bagging</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -8435,18 +8375,14 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>pr-auc</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>0.725</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>0.008999999999999999</v>
       </c>
     </row>
     <row r="14">
@@ -8462,7 +8398,7 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Best of 10 sklearn/XGBoost models on 31 RDKit descriptors</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
@@ -8472,18 +8408,14 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>pr-auc</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>0.388</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>0.05</v>
       </c>
     </row>
     <row r="15">
@@ -8499,7 +8431,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Best of 10 sklearn/XGBoost models on 31 RDKit descriptors</t>
+          <t>AdaBoost</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -8509,18 +8441,14 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>pr-auc</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>0.015</v>
       </c>
     </row>
     <row r="16">
@@ -8536,7 +8464,7 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Best of 10 sklearn/XGBoost models on 31 RDKit descriptors</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -8546,18 +8474,14 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G16" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>0.596</v>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>0.026</v>
       </c>
     </row>
     <row r="17">
@@ -8573,7 +8497,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Best of 10 sklearn/XGBoost models on 31 RDKit descriptors</t>
+          <t>AdaBoost</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -8583,18 +8507,14 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>spearman</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>0.193</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>0.03</v>
       </c>
     </row>
     <row r="18">
@@ -8610,7 +8530,7 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Best of 10 sklearn/XGBoost models on 31 RDKit descriptors</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
@@ -8620,18 +8540,14 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>spearman</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>0.325</v>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>0.039</v>
       </c>
     </row>
     <row r="19">
@@ -8647,7 +8563,7 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Best of 10 sklearn/XGBoost models on 31 RDKit descriptors</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -8657,18 +8573,14 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>spearman</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="n">
+        <v>0.454</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>0.038</v>
       </c>
     </row>
     <row r="20">
@@ -8684,7 +8596,7 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Best of 10 sklearn/XGBoost models on 31 RDKit descriptors</t>
+          <t>ExtraTrees</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
@@ -8694,18 +8606,14 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>mae</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>0.655</v>
+      </c>
+      <c r="G20" s="3" t="n">
+        <v>0.005</v>
       </c>
     </row>
     <row r="21">
@@ -8721,7 +8629,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Best of 10 sklearn/XGBoost models on 31 RDKit descriptors</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -8731,18 +8639,14 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>0.825</v>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>0.024</v>
       </c>
     </row>
     <row r="22">
@@ -8758,7 +8662,7 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Best of 10 sklearn/XGBoost models on 31 RDKit descriptors</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
@@ -8768,18 +8672,14 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G22" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="n">
+        <v>0.788</v>
+      </c>
+      <c r="G22" s="3" t="n">
+        <v>0.008</v>
       </c>
     </row>
     <row r="23">
@@ -8795,7 +8695,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Best of 10 sklearn/XGBoost models on 31 RDKit descriptors</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -8805,18 +8705,14 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G23" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="n">
+        <v>0.882</v>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>0.01</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
finished calicoboost for real and updated results for real
</commit_message>
<xml_diff>
--- a/results/benchmark_results.xlsx
+++ b/results/benchmark_results.xlsx
@@ -8805,18 +8805,14 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>mae</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>0.269</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>0.004</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
added best hyperparameters during validation training to all datasets
</commit_message>
<xml_diff>
--- a/results/benchmark_results.xlsx
+++ b/results/benchmark_results.xlsx
@@ -4010,7 +4010,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -4020,6 +4020,7 @@
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4058,6 +4059,11 @@
           <t>std</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>best_hyperparams</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -4091,6 +4097,11 @@
       <c r="G2" s="3" t="n">
         <v>0.011</v>
       </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>n_estimators=50, max_depth=None</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -4124,6 +4135,11 @@
       <c r="G3" s="2" t="n">
         <v>0.007</v>
       </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>n_estimators=200, max_depth=None</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -4157,6 +4173,11 @@
       <c r="G4" s="3" t="n">
         <v>0.005</v>
       </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>n_estimators=200, max_depth=10</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -4190,6 +4211,11 @@
       <c r="G5" s="2" t="n">
         <v>0.025</v>
       </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>n_estimators=200, max_depth=10</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -4223,6 +4249,11 @@
       <c r="G6" s="3" t="n">
         <v>0.002</v>
       </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>n_estimators=200, max_depth=None</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -4256,6 +4287,11 @@
       <c r="G7" s="2" t="n">
         <v>0.004</v>
       </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>n_estimators=200, max_depth=None</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -4289,6 +4325,11 @@
       <c r="G8" s="3" t="n">
         <v>0.008999999999999999</v>
       </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>n_estimators=50, max_depth=None</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -4322,6 +4363,11 @@
       <c r="G9" s="2" t="n">
         <v>0.06900000000000001</v>
       </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>n_estimators=100, max_depth=None</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -4355,6 +4401,11 @@
       <c r="G10" s="3" t="n">
         <v>0.031</v>
       </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>n_estimators=200, max_depth=10</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -4388,6 +4439,11 @@
       <c r="G11" s="2" t="n">
         <v>0.004</v>
       </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>n_estimators=200, max_depth=10</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -4421,6 +4477,11 @@
       <c r="G12" s="3" t="n">
         <v>0.001</v>
       </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>n_estimators=200, max_depth=None</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -4454,6 +4515,11 @@
       <c r="G13" s="2" t="n">
         <v>0.002</v>
       </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>n_estimators=200, max_depth=None</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -4487,6 +4553,11 @@
       <c r="G14" s="3" t="n">
         <v>0.023</v>
       </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>n_estimators=200, max_depth=None</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -4520,6 +4591,11 @@
       <c r="G15" s="2" t="n">
         <v>0.006</v>
       </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>n_estimators=200, max_depth=10</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -4553,6 +4629,11 @@
       <c r="G16" s="3" t="n">
         <v>0.01</v>
       </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>n_estimators=100, max_depth=None</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -4586,6 +4667,11 @@
       <c r="G17" s="2" t="n">
         <v>0.027</v>
       </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>n_estimators=50, max_depth=None</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -4619,6 +4705,11 @@
       <c r="G18" s="3" t="n">
         <v>0.017</v>
       </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>n_estimators=100, max_depth=None</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -4652,6 +4743,11 @@
       <c r="G19" s="2" t="n">
         <v>0.008999999999999999</v>
       </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>n_estimators=200, max_depth=None</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -4685,6 +4781,11 @@
       <c r="G20" s="3" t="n">
         <v>0.001</v>
       </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>n_estimators=200, max_depth=None</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -4718,6 +4819,11 @@
       <c r="G21" s="2" t="n">
         <v>0.01</v>
       </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>n_estimators=200, max_depth=None</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -4751,6 +4857,11 @@
       <c r="G22" s="3" t="n">
         <v>0.005</v>
       </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>n_estimators=200, max_depth=None</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -4783,6 +4894,11 @@
       </c>
       <c r="G23" s="2" t="n">
         <v>0.008</v>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>n_estimators=200, max_depth=10</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -4796,7 +4912,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -4806,6 +4922,7 @@
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4844,6 +4961,11 @@
           <t>std</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>best_hyperparams</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -4877,6 +4999,11 @@
       <c r="G2" s="3" t="n">
         <v>0.026</v>
       </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -4910,6 +5037,11 @@
       <c r="G3" s="2" t="n">
         <v>0.013</v>
       </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -4943,6 +5075,11 @@
       <c r="G4" s="3" t="n">
         <v>0.008999999999999999</v>
       </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -4976,6 +5113,11 @@
       <c r="G5" s="2" t="n">
         <v>0.031</v>
       </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -5009,6 +5151,11 @@
       <c r="G6" s="3" t="n">
         <v>0.012</v>
       </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -5042,6 +5189,11 @@
       <c r="G7" s="2" t="n">
         <v>0.011</v>
       </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -5075,6 +5227,11 @@
       <c r="G8" s="3" t="n">
         <v>0.006</v>
       </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -5108,6 +5265,11 @@
       <c r="G9" s="2" t="n">
         <v>0.063</v>
       </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -5141,6 +5303,11 @@
       <c r="G10" s="3" t="n">
         <v>0.03</v>
       </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -5174,6 +5341,11 @@
       <c r="G11" s="2" t="n">
         <v>0.026</v>
       </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -5207,6 +5379,11 @@
       <c r="G12" s="3" t="n">
         <v>0.007</v>
       </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -5240,6 +5417,11 @@
       <c r="G13" s="2" t="n">
         <v>0.003</v>
       </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -5273,6 +5455,11 @@
       <c r="G14" s="3" t="n">
         <v>0.016</v>
       </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -5306,6 +5493,11 @@
       <c r="G15" s="2" t="n">
         <v>0.023</v>
       </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -5339,6 +5531,11 @@
       <c r="G16" s="3" t="n">
         <v>0.01</v>
       </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -5372,6 +5569,11 @@
       <c r="G17" s="2" t="n">
         <v>0.051</v>
       </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -5405,6 +5607,11 @@
       <c r="G18" s="3" t="n">
         <v>0.008999999999999999</v>
       </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -5438,6 +5645,11 @@
       <c r="G19" s="2" t="n">
         <v>0.008</v>
       </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -5471,6 +5683,11 @@
       <c r="G20" s="3" t="n">
         <v>0.012</v>
       </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -5504,6 +5721,11 @@
       <c r="G21" s="2" t="n">
         <v>0.023</v>
       </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -5537,6 +5759,11 @@
       <c r="G22" s="3" t="n">
         <v>0.007</v>
       </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -5569,6 +5796,11 @@
       </c>
       <c r="G23" s="2" t="n">
         <v>0.03</v>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -5582,7 +5814,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -5592,6 +5824,7 @@
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5630,6 +5863,11 @@
           <t>std</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>best_hyperparams</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -5663,6 +5901,11 @@
       <c r="G2" s="3" t="n">
         <v>0.004</v>
       </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>iterations=500, learning_rate=0.1</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -5696,6 +5939,11 @@
       <c r="G3" s="2" t="n">
         <v>0.002</v>
       </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>iterations=1000, learning_rate=0.03</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -5729,6 +5977,11 @@
       <c r="G4" s="3" t="n">
         <v>0.001</v>
       </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>iterations=1000, learning_rate=0.03</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -5762,6 +6015,11 @@
       <c r="G5" s="2" t="n">
         <v>0.005</v>
       </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>iterations=1000, learning_rate=0.03</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -5795,6 +6053,11 @@
       <c r="G6" s="3" t="n">
         <v>0.003</v>
       </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>iterations=2000, learning_rate=0.03</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -5828,6 +6091,11 @@
       <c r="G7" s="2" t="n">
         <v>0.01</v>
       </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>iterations=1000, learning_rate=0.03</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -5861,6 +6129,11 @@
       <c r="G8" s="3" t="n">
         <v>0.002</v>
       </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>iterations=1000, learning_rate=0.1</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -5894,6 +6167,11 @@
       <c r="G9" s="2" t="n">
         <v>0.046</v>
       </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>iterations=1000, learning_rate=0.03</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -5927,6 +6205,11 @@
       <c r="G10" s="3" t="n">
         <v>0.013</v>
       </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>iterations=1000, learning_rate=0.03</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -5960,6 +6243,11 @@
       <c r="G11" s="2" t="n">
         <v>0.007</v>
       </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>iterations=1000, learning_rate=0.03</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -5993,6 +6281,11 @@
       <c r="G12" s="3" t="n">
         <v>0.001</v>
       </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>iterations=2000, learning_rate=0.03</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -6026,6 +6319,11 @@
       <c r="G13" s="2" t="n">
         <v>0.004</v>
       </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>iterations=2000, learning_rate=0.03</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -6059,6 +6357,11 @@
       <c r="G14" s="3" t="n">
         <v>0.015</v>
       </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>iterations=500, learning_rate=0.1</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -6092,6 +6395,11 @@
       <c r="G15" s="2" t="n">
         <v>0.006</v>
       </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>iterations=1000, learning_rate=0.1</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -6125,6 +6433,11 @@
       <c r="G16" s="3" t="n">
         <v>0.008999999999999999</v>
       </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>iterations=2000, learning_rate=0.03</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -6158,6 +6471,11 @@
       <c r="G17" s="2" t="n">
         <v>0.027</v>
       </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>iterations=1000, learning_rate=0.03</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -6191,6 +6509,11 @@
       <c r="G18" s="3" t="n">
         <v>0.019</v>
       </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>iterations=1000, learning_rate=0.1</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -6224,6 +6547,11 @@
       <c r="G19" s="2" t="n">
         <v>0.021</v>
       </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>iterations=1000, learning_rate=0.1</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -6257,6 +6585,11 @@
       <c r="G20" s="3" t="n">
         <v>0.004</v>
       </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>iterations=1000, learning_rate=0.1</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -6290,6 +6623,11 @@
       <c r="G21" s="2" t="n">
         <v>0.004</v>
       </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>iterations=1000, learning_rate=0.03</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -6323,6 +6661,11 @@
       <c r="G22" s="3" t="n">
         <v>0.003</v>
       </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>iterations=2000, learning_rate=0.03</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -6355,6 +6698,11 @@
       </c>
       <c r="G23" s="2" t="n">
         <v>0.005</v>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>iterations=1000, learning_rate=0.03</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -6368,7 +6716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -6378,6 +6726,7 @@
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6416,6 +6765,11 @@
           <t>std</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>best_hyperparams</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -6449,6 +6803,11 @@
       <c r="G2" s="3" t="n">
         <v>0.032</v>
       </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>lr=0.001, epochs=20</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -6482,6 +6841,11 @@
       <c r="G3" s="2" t="n">
         <v>0.002</v>
       </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>lr=0.001, epochs=20</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -6515,6 +6879,11 @@
       <c r="G4" s="3" t="n">
         <v>0.005</v>
       </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>lr=0.001, epochs=20</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -6548,6 +6917,11 @@
       <c r="G5" s="2" t="n">
         <v>0.027</v>
       </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>lr=0.001, epochs=20</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -6581,6 +6955,11 @@
       <c r="G6" s="3" t="n">
         <v>0.008999999999999999</v>
       </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>lr=0.001, epochs=20</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -6614,6 +6993,11 @@
       <c r="G7" s="2" t="n">
         <v>0.024</v>
       </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>lr=0.0001, epochs=30</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -6647,6 +7031,11 @@
       <c r="G8" s="3" t="n">
         <v>0.006</v>
       </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>lr=0.001, epochs=20</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -6680,6 +7069,11 @@
       <c r="G9" s="2" t="n">
         <v>0.239</v>
       </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>lr=0.001, epochs=20</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -6713,6 +7107,11 @@
       <c r="G10" s="3" t="n">
         <v>0.013</v>
       </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>lr=0.001, epochs=20</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -6746,6 +7145,11 @@
       <c r="G11" s="2" t="n">
         <v>0.001</v>
       </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>lr=0.0001, epochs=30</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -6779,6 +7183,11 @@
       <c r="G12" s="3" t="n">
         <v>0.001</v>
       </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>lr=0.0001, epochs=30</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -6812,6 +7221,11 @@
       <c r="G13" s="2" t="n">
         <v>0.002</v>
       </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>lr=0.0001, epochs=30</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -6845,6 +7259,11 @@
       <c r="G14" s="3" t="n">
         <v>0.032</v>
       </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>lr=0.0001, epochs=30</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -6878,6 +7297,11 @@
       <c r="G15" s="2" t="n">
         <v>0.016</v>
       </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>lr=0.001, epochs=20</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -6911,6 +7335,11 @@
       <c r="G16" s="3" t="n">
         <v>0.011</v>
       </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>lr=0.001, epochs=20</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -6944,6 +7373,11 @@
       <c r="G17" s="2" t="n">
         <v>0.202</v>
       </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>lr=0.0001, epochs=30</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -6977,6 +7411,11 @@
       <c r="G18" s="3" t="n">
         <v>0.019</v>
       </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>lr=0.001, epochs=20</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -7010,6 +7449,11 @@
       <c r="G19" s="2" t="n">
         <v>0.014</v>
       </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>lr=0.001, epochs=20</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -7043,6 +7487,11 @@
       <c r="G20" s="3" t="n">
         <v>0.026</v>
       </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>lr=0.0001, epochs=30</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -7076,6 +7525,11 @@
       <c r="G21" s="2" t="n">
         <v>0.011</v>
       </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>lr=0.001, epochs=20</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -7109,6 +7563,11 @@
       <c r="G22" s="3" t="n">
         <v>0.005</v>
       </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>lr=0.001, epochs=20</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -7141,6 +7600,11 @@
       </c>
       <c r="G23" s="2" t="n">
         <v>0.008</v>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>lr=0.001, epochs=20</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -7154,7 +7618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -7164,6 +7628,7 @@
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7202,6 +7667,11 @@
           <t>std</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>best_hyperparams</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -7235,6 +7705,11 @@
       <c r="G2" s="3" t="n">
         <v>0.006</v>
       </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>lr=0.0005, epochs=50</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -7268,6 +7743,11 @@
       <c r="G3" s="2" t="n">
         <v>0.002</v>
       </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>lr=0.0005, epochs=50</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -7301,6 +7781,11 @@
       <c r="G4" s="3" t="n">
         <v>0.003</v>
       </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>lr=0.0005, epochs=50</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -7334,6 +7819,11 @@
       <c r="G5" s="2" t="n">
         <v>0.025</v>
       </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>lr=0.0005, epochs=50</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -7367,6 +7857,11 @@
       <c r="G6" s="3" t="n">
         <v>0.017</v>
       </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>lr=0.0005, epochs=50</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -7400,6 +7895,11 @@
       <c r="G7" s="2" t="n">
         <v>0.021</v>
       </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>lr=0.001, epochs=20</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -7433,6 +7933,11 @@
       <c r="G8" s="3" t="n">
         <v>0.004</v>
       </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>lr=0.0005, epochs=50</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -7466,6 +7971,11 @@
       <c r="G9" s="2" t="n">
         <v>0.654</v>
       </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>lr=0.0005, epochs=50</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -7499,6 +8009,11 @@
       <c r="G10" s="3" t="n">
         <v>0.172</v>
       </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>lr=0.0001, epochs=30</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -7532,6 +8047,11 @@
       <c r="G11" s="2" t="n">
         <v>0.008</v>
       </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>lr=0.0005, epochs=50</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -7565,6 +8085,11 @@
       <c r="G12" s="3" t="n">
         <v>0.003</v>
       </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>lr=0.0005, epochs=50</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -7598,6 +8123,11 @@
       <c r="G13" s="2" t="n">
         <v>0.015</v>
       </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>lr=0.0005, epochs=50</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -7631,6 +8161,11 @@
       <c r="G14" s="3" t="n">
         <v>0.007</v>
       </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>lr=0.0005, epochs=50</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -7664,6 +8199,11 @@
       <c r="G15" s="2" t="n">
         <v>0.025</v>
       </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>lr=0.0005, epochs=50</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -7697,6 +8237,11 @@
       <c r="G16" s="3" t="n">
         <v>0.011</v>
       </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>lr=0.0005, epochs=50</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -7730,6 +8275,11 @@
       <c r="G17" s="2" t="n">
         <v>0.039</v>
       </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>lr=0.0005, epochs=50</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -7763,6 +8313,11 @@
       <c r="G18" s="3" t="n">
         <v>0.039</v>
       </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>lr=0.0005, epochs=50</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -7796,6 +8351,11 @@
       <c r="G19" s="2" t="n">
         <v>0.023</v>
       </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>lr=0.0005, epochs=50</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -7829,6 +8389,11 @@
       <c r="G20" s="3" t="n">
         <v>0.024</v>
       </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>lr=0.0005, epochs=50</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -7862,6 +8427,11 @@
       <c r="G21" s="2" t="n">
         <v>0.007</v>
       </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>lr=0.001, epochs=20</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -7895,6 +8465,11 @@
       <c r="G22" s="3" t="n">
         <v>0.004</v>
       </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>lr=0.0005, epochs=50</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -7927,6 +8502,11 @@
       </c>
       <c r="G23" s="2" t="n">
         <v>0.007</v>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>lr=0.0005, epochs=50</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -7940,7 +8520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -7950,6 +8530,7 @@
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7988,6 +8569,11 @@
           <t>std</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>best_hyperparams</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -8021,6 +8607,11 @@
       <c r="G2" s="3" t="n">
         <v>0.083</v>
       </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>Bagging: n_estimators=20, max_samples=1.0</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -8054,6 +8645,11 @@
       <c r="G3" s="2" t="n">
         <v>0.006</v>
       </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Bagging: n_estimators=20, max_samples=0.5</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -8087,6 +8683,11 @@
       <c r="G4" s="3" t="n">
         <v>0.008</v>
       </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>RandomForest: n_estimators=200, max_depth=None</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -8120,6 +8721,11 @@
       <c r="G5" s="2" t="n">
         <v>0.012</v>
       </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>XGBoost: n_estimators=100, max_depth=7, learning_rate=0.1</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -8153,6 +8759,11 @@
       <c r="G6" s="3" t="n">
         <v>0.004</v>
       </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>Bagging: n_estimators=50, max_samples=1.0</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -8186,6 +8797,11 @@
       <c r="G7" s="2" t="n">
         <v>0.011</v>
       </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>XGBoost: n_estimators=100, max_depth=5, learning_rate=0.1</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -8219,6 +8835,11 @@
       <c r="G8" s="3" t="n">
         <v>0.017</v>
       </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>XGBoost: n_estimators=100, max_depth=5, learning_rate=0.1</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -8252,6 +8873,11 @@
       <c r="G9" s="2" t="n">
         <v>0.276</v>
       </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Bagging: n_estimators=20, max_samples=0.5</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -8285,6 +8911,11 @@
       <c r="G10" s="3" t="n">
         <v>0.014</v>
       </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>AdaBoost: n_estimators=100, learning_rate=0.01</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -8318,6 +8949,11 @@
       <c r="G11" s="2" t="n">
         <v>0.021</v>
       </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>XGBoost: n_estimators=200, max_depth=7, learning_rate=0.05</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -8351,6 +8987,11 @@
       <c r="G12" s="3" t="n">
         <v>0.003</v>
       </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>GradientBoosting: n_estimators=100, max_depth=5, learning_rate=0.1</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -8384,6 +9025,11 @@
       <c r="G13" s="2" t="n">
         <v>0.008999999999999999</v>
       </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>XGBoost: n_estimators=200, max_depth=7, learning_rate=0.05</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -8417,6 +9063,11 @@
       <c r="G14" s="3" t="n">
         <v>0.05</v>
       </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>GradientBoosting: n_estimators=100, max_depth=5, learning_rate=0.1</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -8450,6 +9101,11 @@
       <c r="G15" s="2" t="n">
         <v>0.015</v>
       </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>LogisticRegression: C=100</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -8483,6 +9139,11 @@
       <c r="G16" s="3" t="n">
         <v>0.026</v>
       </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>XGBoost: n_estimators=100, max_depth=5, learning_rate=0.1</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -8516,6 +9177,11 @@
       <c r="G17" s="2" t="n">
         <v>0.03</v>
       </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Bagging: n_estimators=10, max_samples=0.5</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -8549,6 +9215,11 @@
       <c r="G18" s="3" t="n">
         <v>0.039</v>
       </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>ExtraTrees: n_estimators=200, max_depth=10</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -8582,6 +9253,11 @@
       <c r="G19" s="2" t="n">
         <v>0.038</v>
       </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Bagging: n_estimators=50, max_samples=1.0</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -8615,6 +9291,11 @@
       <c r="G20" s="3" t="n">
         <v>0.005</v>
       </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>ExtraTrees: n_estimators=200, max_depth=None</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -8648,6 +9329,11 @@
       <c r="G21" s="2" t="n">
         <v>0.024</v>
       </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>ExtraTrees: n_estimators=200, max_depth=10</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -8681,6 +9367,11 @@
       <c r="G22" s="3" t="n">
         <v>0.008</v>
       </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>XGBoost: n_estimators=200, max_depth=7, learning_rate=0.05</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -8713,6 +9404,11 @@
       </c>
       <c r="G23" s="2" t="n">
         <v>0.01</v>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>RandomForest: n_estimators=200, max_depth=None</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -8726,7 +9422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -8736,6 +9432,7 @@
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8781,6 +9478,11 @@
           <t>std</t>
         </is>
       </c>
+      <c r="H3" s="1" t="inlineStr">
+        <is>
+          <t>best_hyperparams</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -8814,6 +9516,11 @@
       <c r="G4" s="3" t="n">
         <v>0.004</v>
       </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>n_estimators=1000, learning_rate=0.03, max_depth=6, subsample=0.8, colsample_bytree=0.8, min_child_weight=3, reg_alpha=0.1, reg_lambda=1.0, random_state=42, verbosity=0</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -8851,6 +9558,11 @@
           <t>N/A</t>
         </is>
       </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -8888,6 +9600,11 @@
           <t>N/A</t>
         </is>
       </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -8925,6 +9642,11 @@
           <t>N/A</t>
         </is>
       </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -8962,6 +9684,11 @@
           <t>N/A</t>
         </is>
       </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -8999,6 +9726,11 @@
           <t>N/A</t>
         </is>
       </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -9036,6 +9768,11 @@
           <t>N/A</t>
         </is>
       </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -9073,6 +9810,11 @@
           <t>N/A</t>
         </is>
       </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
@@ -9110,6 +9852,11 @@
           <t>N/A</t>
         </is>
       </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -9147,6 +9894,11 @@
           <t>N/A</t>
         </is>
       </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
@@ -9184,6 +9936,11 @@
           <t>N/A</t>
         </is>
       </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -9221,6 +9978,11 @@
           <t>N/A</t>
         </is>
       </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
@@ -9258,6 +10020,11 @@
           <t>N/A</t>
         </is>
       </c>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -9295,6 +10062,11 @@
           <t>N/A</t>
         </is>
       </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
@@ -9332,6 +10104,11 @@
           <t>N/A</t>
         </is>
       </c>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -9369,6 +10146,11 @@
           <t>N/A</t>
         </is>
       </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
@@ -9406,6 +10188,11 @@
           <t>N/A</t>
         </is>
       </c>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -9443,6 +10230,11 @@
           <t>N/A</t>
         </is>
       </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
@@ -9480,6 +10272,11 @@
           <t>N/A</t>
         </is>
       </c>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
@@ -9517,6 +10314,11 @@
           <t>N/A</t>
         </is>
       </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
@@ -9554,6 +10356,11 @@
           <t>N/A</t>
         </is>
       </c>
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
@@ -9587,6 +10394,11 @@
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>

</xml_diff>

<commit_message>
further improvements to the result generation
</commit_message>
<xml_diff>
--- a/results/benchmark_results.xlsx
+++ b/results/benchmark_results.xlsx
@@ -5001,7 +5001,7 @@
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>combo selected: morgan_1024+xgb (no hyperparams tuned)</t>
         </is>
       </c>
     </row>
@@ -5039,7 +5039,7 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>combo selected: morgan_2048+rf_100 (no hyperparams tuned)</t>
         </is>
       </c>
     </row>
@@ -5077,7 +5077,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>combo selected: morgan_2048+rf_200 (no hyperparams tuned)</t>
         </is>
       </c>
     </row>
@@ -5115,7 +5115,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>combo selected: morgan_2048+rf_100 (no hyperparams tuned)</t>
         </is>
       </c>
     </row>
@@ -5153,7 +5153,7 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>combo selected: morgan_2048+xgb (no hyperparams tuned)</t>
         </is>
       </c>
     </row>
@@ -5191,7 +5191,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>combo selected: morgan_2048+xgb (no hyperparams tuned)</t>
         </is>
       </c>
     </row>
@@ -5229,7 +5229,7 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>combo selected: morgan_1024+rf_100 (no hyperparams tuned)</t>
         </is>
       </c>
     </row>
@@ -5267,7 +5267,7 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>combo selected: morgan_1024+xgb (no hyperparams tuned)</t>
         </is>
       </c>
     </row>
@@ -5305,7 +5305,7 @@
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>combo selected: morgan_2048+xgb (no hyperparams tuned)</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>combo selected: morgan_2048+xgb (no hyperparams tuned)</t>
         </is>
       </c>
     </row>
@@ -5381,7 +5381,7 @@
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>combo selected: morgan_2048+rf_200 (no hyperparams tuned)</t>
         </is>
       </c>
     </row>
@@ -5419,7 +5419,7 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>combo selected: morgan_2048+rf_200 (no hyperparams tuned)</t>
         </is>
       </c>
     </row>
@@ -5457,7 +5457,7 @@
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>combo selected: morgan_1024+xgb (no hyperparams tuned)</t>
         </is>
       </c>
     </row>
@@ -5495,7 +5495,7 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>combo selected: morgan_2048+xgb (no hyperparams tuned)</t>
         </is>
       </c>
     </row>
@@ -5533,7 +5533,7 @@
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>combo selected: morgan_1024+rf_100 (no hyperparams tuned)</t>
         </is>
       </c>
     </row>
@@ -5571,7 +5571,7 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>combo selected: morgan_1024+rf_200 (no hyperparams tuned)</t>
         </is>
       </c>
     </row>
@@ -5609,7 +5609,7 @@
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>combo selected: morgan_2048+rf_100 (no hyperparams tuned)</t>
         </is>
       </c>
     </row>
@@ -5647,7 +5647,7 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>combo selected: morgan_2048+rf_200 (no hyperparams tuned)</t>
         </is>
       </c>
     </row>
@@ -5685,7 +5685,7 @@
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>combo selected: morgan_2048+rf_200 (no hyperparams tuned)</t>
         </is>
       </c>
     </row>
@@ -5723,7 +5723,7 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>combo selected: morgan_2048+xgb (no hyperparams tuned)</t>
         </is>
       </c>
     </row>
@@ -5761,7 +5761,7 @@
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>combo selected: morgan_2048+xgb (no hyperparams tuned)</t>
         </is>
       </c>
     </row>
@@ -5799,7 +5799,7 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>combo selected: morgan_2048+rf_200 (no hyperparams tuned)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
base boosting results added
</commit_message>
<xml_diff>
--- a/results/benchmark_results.xlsx
+++ b/results/benchmark_results.xlsx
@@ -10415,51 +10415,894 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="90" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
-        <is>
-          <t>❌ BaseBoosting — Could Not Run</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>benchmark</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>algorithm</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>task_type</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>leaderboard_metric</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>score</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>std</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>best_hyperparams</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="inlineStr">
-        <is>
-          <t>Reason: olorenchemengine (OCE) is not available as a prebuilt wheel on PyPI.</t>
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>caco2_wang</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>BaseBoosting</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Gradient-boosted ensemble of 3 RFs (Morgan + RDKit2D + GIN)</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>regression</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>mae</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>0.318</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
-        <is>
-          <t>Installation requires cloning from GitHub (github.com/Oloren-AI/olorenchemengine),</t>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>hia_hou</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>BaseBoosting</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Gradient-boosted ensemble of 3 RFs (Morgan + RDKit2D + GIN)</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>binary</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>0.972</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
-        <is>
-          <t>which is blocked by the company server firewall.</t>
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>pgp_broccatelli</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>BaseBoosting</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Gradient-boosted ensemble of 3 RFs (Morgan + RDKit2D + GIN)</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>binary</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>0.9340000000000001</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t>All three install methods attempted: pip, Tsinghua mirror, git clone — all failed.</t>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>bioavailability_ma</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>BaseBoosting</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Gradient-boosted ensemble of 3 RFs (Morgan + RDKit2D + GIN)</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>binary</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>0.6909999999999999</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>BaseBoosting can only be run on a machine with unrestricted internet access to GitHub.</t>
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>lipophilicity_astrazeneca</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>BaseBoosting</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Gradient-boosted ensemble of 3 RFs (Morgan + RDKit2D + GIN)</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>regression</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>mae</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>0.6850000000000001</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>solubility_aqsoldb</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>BaseBoosting</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Gradient-boosted ensemble of 3 RFs (Morgan + RDKit2D + GIN)</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>regression</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>mae</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>bbb_martins</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>BaseBoosting</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Gradient-boosted ensemble of 3 RFs (Morgan + RDKit2D + GIN)</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>binary</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>0.915</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>ppbr_az</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>BaseBoosting</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Gradient-boosted ensemble of 3 RFs (Morgan + RDKit2D + GIN)</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>regression</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>mae</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>0.017</v>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>vdss_lombardo</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>BaseBoosting</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Gradient-boosted ensemble of 3 RFs (Morgan + RDKit2D + GIN)</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>regression</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>spearman</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>0.535</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>cyp2d6_veith</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>BaseBoosting</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Gradient-boosted ensemble of 3 RFs (Morgan + RDKit2D + GIN)</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>binary</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>pr-auc</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>0.695</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>cyp3a4_veith</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>BaseBoosting</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Gradient-boosted ensemble of 3 RFs (Morgan + RDKit2D + GIN)</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>binary</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>pr-auc</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>0.861</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>cyp2c9_veith</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>BaseBoosting</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Gradient-boosted ensemble of 3 RFs (Morgan + RDKit2D + GIN)</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>binary</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>pr-auc</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>0.772</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>cyp2c9_substrate_carbonmangels</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>BaseBoosting</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Gradient-boosted ensemble of 3 RFs (Morgan + RDKit2D + GIN)</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>binary</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>pr-auc</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>0.411</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>cyp2d6_substrate_carbonmangels</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>BaseBoosting</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Gradient-boosted ensemble of 3 RFs (Morgan + RDKit2D + GIN)</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>binary</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>pr-auc</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>0.702</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>cyp3a4_substrate_carbonmangels</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>BaseBoosting</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Gradient-boosted ensemble of 3 RFs (Morgan + RDKit2D + GIN)</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>binary</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>half_life_obach</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>BaseBoosting</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Gradient-boosted ensemble of 3 RFs (Morgan + RDKit2D + GIN)</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>regression</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>spearman</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>0.407</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>clearance_hepatocyte_az</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>BaseBoosting</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Gradient-boosted ensemble of 3 RFs (Morgan + RDKit2D + GIN)</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>regression</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>spearman</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>0.476</v>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>clearance_microsome_az</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>BaseBoosting</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Gradient-boosted ensemble of 3 RFs (Morgan + RDKit2D + GIN)</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>regression</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>spearman</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>ld50_zhu</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>BaseBoosting</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Gradient-boosted ensemble of 3 RFs (Morgan + RDKit2D + GIN)</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>regression</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>mae</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>0.644</v>
+      </c>
+      <c r="G20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>herg</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>BaseBoosting</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Gradient-boosted ensemble of 3 RFs (Morgan + RDKit2D + GIN)</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>binary</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>0.851</v>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>ames</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>BaseBoosting</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Gradient-boosted ensemble of 3 RFs (Morgan + RDKit2D + GIN)</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>binary</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="n">
+        <v>0.853</v>
+      </c>
+      <c r="G22" s="3" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>dili</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>BaseBoosting</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Gradient-boosted ensemble of 3 RFs (Morgan + RDKit2D + GIN)</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>binary</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>roc-auc</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="n">
+        <v>0.926</v>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>

</xml_diff>